<commit_message>
Add distinct sample imports and count duplicate records before saving
</commit_message>
<xml_diff>
--- a/assets/templates/MSME_Import_Blank.xlsx
+++ b/assets/templates/MSME_Import_Blank.xlsx
@@ -375,6 +375,13 @@
     <col min="41" max="41" width="22" customWidth="1"/>
     <col min="42" max="42" width="22" customWidth="1"/>
     <col min="43" max="43" width="22" customWidth="1"/>
+    <col min="44" max="44" width="28" customWidth="1"/>
+    <col min="45" max="45" width="28" customWidth="1"/>
+    <col min="46" max="46" width="28" customWidth="1"/>
+    <col min="47" max="47" width="28" customWidth="1"/>
+    <col min="48" max="48" width="28" customWidth="1"/>
+    <col min="49" max="49" width="28" customWidth="1"/>
+    <col min="50" max="50" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="66" customHeight="1">
@@ -591,6 +598,41 @@
       <c r="AQ1" t="inlineStr" s="8">
         <is>
           <t>Challenges Encountered</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr" s="8">
+        <is>
+          <t>Night Market Stall/Booth No.</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr" s="8">
+        <is>
+          <t>Date Started</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr" s="8">
+        <is>
+          <t>Night Market Two-Day Earnings</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr" s="8">
+        <is>
+          <t>Night Market Total Earnings</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr" s="8">
+        <is>
+          <t>Website/Social Media</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr" s="8">
+        <is>
+          <t>Email Address</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr" s="8">
+        <is>
+          <t>Owner Contact Number</t>
         </is>
       </c>
     </row>
@@ -638,6 +680,13 @@
       <c r="AO2" s="0"/>
       <c r="AP2" s="0"/>
       <c r="AQ2" s="0"/>
+      <c r="AR2" s="0"/>
+      <c r="AS2" s="0"/>
+      <c r="AT2" s="0"/>
+      <c r="AU2" s="0"/>
+      <c r="AV2" s="0"/>
+      <c r="AW2" s="0"/>
+      <c r="AX2" s="0"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="0"/>
@@ -683,6 +732,13 @@
       <c r="AO3" s="0"/>
       <c r="AP3" s="0"/>
       <c r="AQ3" s="0"/>
+      <c r="AR3" s="0"/>
+      <c r="AS3" s="0"/>
+      <c r="AT3" s="0"/>
+      <c r="AU3" s="0"/>
+      <c r="AV3" s="0"/>
+      <c r="AW3" s="0"/>
+      <c r="AX3" s="0"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="0"/>
@@ -728,6 +784,13 @@
       <c r="AO4" s="0"/>
       <c r="AP4" s="0"/>
       <c r="AQ4" s="0"/>
+      <c r="AR4" s="0"/>
+      <c r="AS4" s="0"/>
+      <c r="AT4" s="0"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
+      <c r="AW4" s="0"/>
+      <c r="AX4" s="0"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="0"/>
@@ -773,6 +836,13 @@
       <c r="AO5" s="0"/>
       <c r="AP5" s="0"/>
       <c r="AQ5" s="0"/>
+      <c r="AR5" s="0"/>
+      <c r="AS5" s="0"/>
+      <c r="AT5" s="0"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
+      <c r="AW5" s="0"/>
+      <c r="AX5" s="0"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="0"/>
@@ -818,6 +888,13 @@
       <c r="AO6" s="0"/>
       <c r="AP6" s="0"/>
       <c r="AQ6" s="0"/>
+      <c r="AR6" s="0"/>
+      <c r="AS6" s="0"/>
+      <c r="AT6" s="0"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
+      <c r="AW6" s="0"/>
+      <c r="AX6" s="0"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="0"/>
@@ -863,6 +940,13 @@
       <c r="AO7" s="0"/>
       <c r="AP7" s="0"/>
       <c r="AQ7" s="0"/>
+      <c r="AR7" s="0"/>
+      <c r="AS7" s="0"/>
+      <c r="AT7" s="0"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
+      <c r="AW7" s="0"/>
+      <c r="AX7" s="0"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="0"/>
@@ -908,6 +992,13 @@
       <c r="AO8" s="0"/>
       <c r="AP8" s="0"/>
       <c r="AQ8" s="0"/>
+      <c r="AR8" s="0"/>
+      <c r="AS8" s="0"/>
+      <c r="AT8" s="0"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
+      <c r="AW8" s="0"/>
+      <c r="AX8" s="0"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="0"/>
@@ -953,6 +1044,13 @@
       <c r="AO9" s="0"/>
       <c r="AP9" s="0"/>
       <c r="AQ9" s="0"/>
+      <c r="AR9" s="0"/>
+      <c r="AS9" s="0"/>
+      <c r="AT9" s="0"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
+      <c r="AW9" s="0"/>
+      <c r="AX9" s="0"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="0"/>
@@ -998,6 +1096,13 @@
       <c r="AO10" s="0"/>
       <c r="AP10" s="0"/>
       <c r="AQ10" s="0"/>
+      <c r="AR10" s="0"/>
+      <c r="AS10" s="0"/>
+      <c r="AT10" s="0"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
+      <c r="AW10" s="0"/>
+      <c r="AX10" s="0"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="0"/>
@@ -1043,6 +1148,13 @@
       <c r="AO11" s="0"/>
       <c r="AP11" s="0"/>
       <c r="AQ11" s="0"/>
+      <c r="AR11" s="0"/>
+      <c r="AS11" s="0"/>
+      <c r="AT11" s="0"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
+      <c r="AW11" s="0"/>
+      <c r="AX11" s="0"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="0"/>
@@ -1088,6 +1200,13 @@
       <c r="AO12" s="0"/>
       <c r="AP12" s="0"/>
       <c r="AQ12" s="0"/>
+      <c r="AR12" s="0"/>
+      <c r="AS12" s="0"/>
+      <c r="AT12" s="0"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
+      <c r="AW12" s="0"/>
+      <c r="AX12" s="0"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="0"/>
@@ -1133,6 +1252,13 @@
       <c r="AO13" s="0"/>
       <c r="AP13" s="0"/>
       <c r="AQ13" s="0"/>
+      <c r="AR13" s="0"/>
+      <c r="AS13" s="0"/>
+      <c r="AT13" s="0"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
+      <c r="AW13" s="0"/>
+      <c r="AX13" s="0"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="0"/>
@@ -1178,6 +1304,13 @@
       <c r="AO14" s="0"/>
       <c r="AP14" s="0"/>
       <c r="AQ14" s="0"/>
+      <c r="AR14" s="0"/>
+      <c r="AS14" s="0"/>
+      <c r="AT14" s="0"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
+      <c r="AW14" s="0"/>
+      <c r="AX14" s="0"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="0"/>
@@ -1223,6 +1356,13 @@
       <c r="AO15" s="0"/>
       <c r="AP15" s="0"/>
       <c r="AQ15" s="0"/>
+      <c r="AR15" s="0"/>
+      <c r="AS15" s="0"/>
+      <c r="AT15" s="0"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
+      <c r="AW15" s="0"/>
+      <c r="AX15" s="0"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="0"/>
@@ -1268,6 +1408,13 @@
       <c r="AO16" s="0"/>
       <c r="AP16" s="0"/>
       <c r="AQ16" s="0"/>
+      <c r="AR16" s="0"/>
+      <c r="AS16" s="0"/>
+      <c r="AT16" s="0"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
+      <c r="AW16" s="0"/>
+      <c r="AX16" s="0"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="0"/>
@@ -1313,6 +1460,13 @@
       <c r="AO17" s="0"/>
       <c r="AP17" s="0"/>
       <c r="AQ17" s="0"/>
+      <c r="AR17" s="0"/>
+      <c r="AS17" s="0"/>
+      <c r="AT17" s="0"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
+      <c r="AW17" s="0"/>
+      <c r="AX17" s="0"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="0"/>
@@ -1358,6 +1512,13 @@
       <c r="AO18" s="0"/>
       <c r="AP18" s="0"/>
       <c r="AQ18" s="0"/>
+      <c r="AR18" s="0"/>
+      <c r="AS18" s="0"/>
+      <c r="AT18" s="0"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
+      <c r="AW18" s="0"/>
+      <c r="AX18" s="0"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="0"/>
@@ -1403,6 +1564,13 @@
       <c r="AO19" s="0"/>
       <c r="AP19" s="0"/>
       <c r="AQ19" s="0"/>
+      <c r="AR19" s="0"/>
+      <c r="AS19" s="0"/>
+      <c r="AT19" s="0"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
+      <c r="AW19" s="0"/>
+      <c r="AX19" s="0"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="0"/>
@@ -1448,6 +1616,13 @@
       <c r="AO20" s="0"/>
       <c r="AP20" s="0"/>
       <c r="AQ20" s="0"/>
+      <c r="AR20" s="0"/>
+      <c r="AS20" s="0"/>
+      <c r="AT20" s="0"/>
+      <c r="AU20" s="0"/>
+      <c r="AV20" s="0"/>
+      <c r="AW20" s="0"/>
+      <c r="AX20" s="0"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="0"/>
@@ -1493,6 +1668,13 @@
       <c r="AO21" s="0"/>
       <c r="AP21" s="0"/>
       <c r="AQ21" s="0"/>
+      <c r="AR21" s="0"/>
+      <c r="AS21" s="0"/>
+      <c r="AT21" s="0"/>
+      <c r="AU21" s="0"/>
+      <c r="AV21" s="0"/>
+      <c r="AW21" s="0"/>
+      <c r="AX21" s="0"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>